<commit_message>
Rename mode column header
</commit_message>
<xml_diff>
--- a/templates/yangi_shablon.xlsx
+++ b/templates/yangi_shablon.xlsx
@@ -1,103 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EMU\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A1C249B-2D6E-4FA9-A1FF-3C011B296E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Шаблон" sheetId="1" r:id="rId1"/>
+    <sheet name="Шаблон" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
-  <si>
-    <t>Номер</t>
-  </si>
-  <si>
-    <t>Компания-получатель</t>
-  </si>
-  <si>
-    <t>ФИО получателя</t>
-  </si>
-  <si>
-    <t>Адрес получателя</t>
-  </si>
-  <si>
-    <t>Телефон получателя</t>
-  </si>
-  <si>
-    <t>Шифр клиента</t>
-  </si>
-  <si>
-    <t>Масса посылки</t>
-  </si>
-  <si>
-    <t>Поручение</t>
-  </si>
-  <si>
-    <t>Количество мест</t>
-  </si>
-  <si>
-    <t>Штрихкод (№ накладной)</t>
-  </si>
-  <si>
-    <t>Компания-отправитель</t>
-  </si>
-  <si>
-    <t>ФИО отправителя</t>
-  </si>
-  <si>
-    <t>Адрес отправителя</t>
-  </si>
-  <si>
-    <t>Телефон отправителя</t>
-  </si>
-  <si>
-    <t>Город-отправитель</t>
-  </si>
-  <si>
-    <t>Город-получатель</t>
-  </si>
-  <si>
-    <t>Оплата получателем</t>
-  </si>
-  <si>
-    <t>True</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
-      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -116,22 +52,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -419,83 +414,123 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="21" customWidth="1"/>
-    <col min="5" max="5" width="23" customWidth="1"/>
-    <col min="6" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="27" customWidth="1"/>
-    <col min="11" max="11" width="25" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
-    <col min="13" max="13" width="22" customWidth="1"/>
-    <col min="14" max="14" width="24" customWidth="1"/>
-    <col min="15" max="15" width="22" customWidth="1"/>
-    <col min="16" max="16" width="21" customWidth="1"/>
-    <col min="17" max="17" width="23" customWidth="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="23" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Номер</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Компания-получатель</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ФИО получателя</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Адрес получателя</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Телефон получателя</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Шифр клиента</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Масса посылки</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Поручение</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Количество мест</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Режим</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Компания-отправитель</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ФИО отправителя</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Адрес отправителя</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Телефон отправителя</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Город-отправитель</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Город-получатель</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Оплата получателем</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="Q2" t="s">
-        <v>17</v>
+    <row r="2">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add package code column setup
</commit_message>
<xml_diff>
--- a/templates/yangi_shablon.xlsx
+++ b/templates/yangi_shablon.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -437,6 +437,7 @@
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="23" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -523,6 +524,11 @@
       <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Оплата получателем</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Код упаковке</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add template command and optional packaging fields
</commit_message>
<xml_diff>
--- a/templates/yangi_shablon.xlsx
+++ b/templates/yangi_shablon.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -437,7 +437,8 @@
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="23" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,6 +528,11 @@
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Тип вложение</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Код упаковке</t>
         </is>

</xml_diff>

<commit_message>
Clear template default payment value
</commit_message>
<xml_diff>
--- a/templates/yangi_shablon.xlsx
+++ b/templates/yangi_shablon.xlsx
@@ -538,13 +538,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
+    <row r="2"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Split Excel schemas for legal customers
</commit_message>
<xml_diff>
--- a/templates/yangi_shablon.xlsx
+++ b/templates/yangi_shablon.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -428,6 +428,8 @@
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="8"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="27" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
@@ -527,18 +529,7 @@
           <t>Оплата получателем</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Тип вложение</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Код упаковке</t>
-        </is>
-      </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add persistent import numbers for Excel exports
</commit_message>
<xml_diff>
--- a/templates/yangi_shablon.xlsx
+++ b/templates/yangi_shablon.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Шаблон" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Шаблон" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -419,10 +419,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
@@ -444,87 +444,92 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Номер</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Компания-получатель</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ФИО получателя</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Адрес получателя</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Телефон получателя</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Шифр клиента</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Масса посылки</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Поручение</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Количество мест</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Режим</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Компания-отправитель</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ФИО отправителя</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Адрес отправителя</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Телефон отправителя</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Город-отправитель</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Город-получатель</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Оплата получателем</t>
         </is>

</xml_diff>